<commit_message>
🔒 [FULL] Daily chip data 2026-08-03 22:55
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -1656,7 +1656,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 🎯 quad 進場 (78.9% alpha): 2308 / 6770 / 2330 +6  |  避開 — 除權息 7 檔: 1465, 1527, 2367 ... | 明日恐處置 6 檔: 3374/4542/4556...  |  訊號: 強偏多 (Q5 81.7%, hot=21)</t>
+          <t>💡 🎯 quad 進場 (78.9% alpha): 2308 / 6770 / 2330 +6  |  避開 — 除權息 7 檔: 1465, 1527, 2367 ... | 明日恐處置 1 檔: 3362  |  訊號: 強偏多 (Q5 81.7%, hot=21)</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
     <row r="37">
       <c r="C37" s="71" t="inlineStr">
         <is>
-          <t>明日恐處置 6 檔 (3374 / 4542 / 4556 ...)</t>
+          <t>明日恐處置 1 檔 (3362)</t>
         </is>
       </c>
     </row>
@@ -30436,7 +30436,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="204" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-03 21:34 TW | 0/23 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-03 22:55 TW | 0/23 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-04 01:49
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -35,6 +35,8 @@
     <numFmt numFmtId="174" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="175" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="176" formatCode="#,##0.00;-#,##0.00"/>
+    <numFmt numFmtId="177" formatCode="0&quot; 檔 +120億 &quot;&quot;(昨5/5d9)&quot;"/>
+    <numFmt numFmtId="178" formatCode="0.0%&quot; 市-960億 &quot;&quot;(昨15/5d16)&quot;"/>
   </numFmts>
   <fonts count="53">
     <font>
@@ -341,7 +343,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="49">
+  <fills count="50">
     <fill>
       <patternFill/>
     </fill>
@@ -585,6 +587,12 @@
         <fgColor rgb="FFD1FAE5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -598,7 +606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="238">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1145,6 +1153,24 @@
     <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1230,12 +1256,12 @@
     <comment ref="D19" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 83.1%
+領頭大戶「張濬安(航海王)」獨佔比 84.0%
   • 領頭金額 104,611 萬
-  • 合計淨買 125,848 萬
+  • 合計淨買 124,595 萬
   • 大戶數 12 位 (名義共識)
 判讀: 名義 12 位大戶共識,
-實質 1 人下注佔 83%,
+實質 1 人下注佔 84%,
 剩餘 11 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1243,9 +1269,9 @@
     <comment ref="D20" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 56.8%
-  • 領頭金額 55,828 萬
-  • 合計淨買 98,358 萬
+領頭大戶「陳族元」獨佔比 56.7%
+  • 領頭金額 55,645 萬
+  • 合計淨買 98,174 萬
   • 大戶數 13 位 (名義共識)
 判讀: 名義 13 位大戶共識,
 實質 1 人下注佔 57%,
@@ -1269,12 +1295,12 @@
     <comment ref="D22" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 57.9%
-  • 領頭金額 24,657 萬
-  • 合計淨買 42,552 萬
+領頭大戶「陳族元」獨佔比 58.8%
+  • 領頭金額 25,491 萬
+  • 合計淨買 43,385 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
-實質 1 人下注佔 58%,
+實質 1 人下注佔 59%,
 剩餘 10 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1295,12 +1321,12 @@
     <comment ref="D24" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳律師」獨佔比 53.6%
+領頭大戶「陳律師」獨佔比 56.6%
   • 領頭金額 15,283 萬
-  • 合計淨買 28,538 萬
+  • 合計淨買 27,020 萬
   • 大戶數 12 位 (名義共識)
 判讀: 名義 12 位大戶共識,
-實質 1 人下注佔 54%,
+實質 1 人下注佔 57%,
 剩餘 11 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1816,7 +1842,7 @@
         </is>
       </c>
       <c r="H16" s="17" t="n">
-        <v>193024</v>
+        <v>175305</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1838,7 +1864,7 @@
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>441946</v>
+        <v>424227</v>
       </c>
     </row>
     <row r="17">
@@ -1867,7 +1893,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>85501</v>
+        <v>85215</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1889,7 +1915,7 @@
         <v>9</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>193870</v>
+        <v>193584</v>
       </c>
     </row>
     <row r="18">
@@ -1926,7 +1952,7 @@
         </is>
       </c>
       <c r="J18" s="18" t="n">
-        <v>52121</v>
+        <v>53420</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1940,7 +1966,7 @@
         <v>10</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>184850</v>
+        <v>186148</v>
       </c>
     </row>
     <row r="19">
@@ -1981,17 +2007,17 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L19" s="18" t="n">
-        <v>3583</v>
+        <v>3049</v>
       </c>
       <c r="M19" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N19" s="17" t="n">
-        <v>125848</v>
+        <v>124595</v>
       </c>
     </row>
     <row r="20">
@@ -2020,7 +2046,7 @@
         </is>
       </c>
       <c r="H20" s="17" t="n">
-        <v>55829</v>
+        <v>55645</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2042,7 +2068,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>98358</v>
+        <v>98174</v>
       </c>
     </row>
     <row r="21">
@@ -2114,7 +2140,7 @@
         <v>11</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
@@ -2122,7 +2148,7 @@
         </is>
       </c>
       <c r="H22" s="17" t="n">
-        <v>24658</v>
+        <v>25491</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2144,7 +2170,7 @@
         <v>8</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>42552</v>
+        <v>43386</v>
       </c>
     </row>
     <row r="23">
@@ -2236,17 +2262,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="L24" s="18" t="n">
-        <v>2399</v>
+        <v>1747</v>
       </c>
       <c r="M24" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>28538</v>
+        <v>27020</v>
       </c>
     </row>
     <row r="25">
@@ -2322,7 +2348,7 @@
         </is>
       </c>
       <c r="G28" s="208" t="n">
-        <v>123.7623</v>
+        <v>121.3232</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
@@ -2331,7 +2357,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C29" s="209" t="n">
+      <c r="C29" s="238" t="n">
         <v>10</v>
       </c>
       <c r="F29" s="22" t="inlineStr">
@@ -2339,8 +2365,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G29" s="210" t="n">
-        <v>0.2294531048392597</v>
+      <c r="G29" s="239" t="n">
+        <v>0.2281411777835858</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2419,11 +2445,11 @@
         </is>
       </c>
       <c r="D35" s="33" t="n">
-        <v>1633313</v>
+        <v>1589585</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>27.1%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2435,7 +2461,7 @@
         </is>
       </c>
       <c r="H35" s="33" t="n">
-        <v>441946</v>
+        <v>424227</v>
       </c>
       <c r="I35" s="212" t="n">
         <v>-0.0227</v>
@@ -2455,7 +2481,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.2%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2487,7 +2513,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2499,7 +2525,7 @@
         </is>
       </c>
       <c r="H37" s="33" t="n">
-        <v>231618</v>
+        <v>231704</v>
       </c>
       <c r="I37" s="213" t="n">
         <v>0.0495</v>
@@ -2519,7 +2545,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.4%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2531,7 +2557,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>193870</v>
+        <v>193584</v>
       </c>
       <c r="I38" s="213" t="n">
         <v>0.0345</v>
@@ -2551,7 +2577,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2563,7 +2589,7 @@
         </is>
       </c>
       <c r="H39" s="33" t="n">
-        <v>184850</v>
+        <v>186148</v>
       </c>
       <c r="I39" s="212" t="n">
         <v>-0.0248</v>
@@ -2979,11 +3005,11 @@
         <v>48</v>
       </c>
       <c r="E60" t="n">
-        <v>5512941</v>
+        <v>5495856</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>陳族元 連續 48 天加碼 2330 (累計 5,512,941 萬)</t>
+          <t>陳族元 連續 48 天加碼 2330 (累計 5,495,856 萬)</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3166,7 @@
         </is>
       </c>
       <c r="C68" s="33" t="n">
-        <v>1490209</v>
+        <v>1448081</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3148,7 +3174,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>200755</v>
+        <v>183670</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3164,10 +3190,10 @@
         </is>
       </c>
       <c r="I68" s="33" t="n">
-        <v>127764</v>
+        <v>127776</v>
       </c>
       <c r="J68" s="214" t="n">
-        <v>0.3132101774207987</v>
+        <v>0.3105319337520347</v>
       </c>
     </row>
     <row r="69">
@@ -5074,7 +5100,7 @@
     <row r="40" ht="22" customHeight="1">
       <c r="C40" s="75" t="inlineStr">
         <is>
-          <t>+124 億 淨買</t>
+          <t>+121 億 淨買</t>
         </is>
       </c>
     </row>
@@ -12240,7 +12266,7 @@
     <row r="1" ht="16.5" customHeight="1">
       <c r="A1" s="110" t="inlineStr">
         <is>
-          <t>⚠️ 本 Excel 無 top-buyer highlight — histock 資料仍是 T-1 (需等到當日盤後晚間 update, 23 次) | attempted=23, success=0</t>
+          <t>⚠️ 部分 top-buyer highlight 缺 (histock: 17/23 = 73% success | fetch_fail=6 stale=0 empty=0)</t>
         </is>
       </c>
       <c r="B1" s="111" t="n"/>
@@ -19431,29 +19457,29 @@
       </c>
       <c r="D190" s="137" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>致茂(2360)</t>
         </is>
       </c>
       <c r="E190" s="138" t="n">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="F190" s="138" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G190" s="138" t="n">
-        <v>19834</v>
+        <v>4080</v>
       </c>
       <c r="H190" s="138" t="n">
-        <v>876</v>
+        <v>3246</v>
       </c>
       <c r="I190" s="138" t="n">
-        <v>18958</v>
+        <v>834</v>
       </c>
       <c r="J190" s="139" t="n">
-        <v>2389.67</v>
+        <v>1942.62</v>
       </c>
       <c r="K190" s="139" t="n">
-        <v>2190.25</v>
+        <v>1909.41</v>
       </c>
       <c r="L190" s="236">
         <f>F190*(K190-J190)</f>
@@ -19466,31 +19492,31 @@
       <c r="C191" s="140" t="n"/>
       <c r="D191" s="137" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E191" s="138" t="n">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="F191" s="138" t="n">
-        <v>48</v>
+        <v>92</v>
       </c>
       <c r="G191" s="138" t="n">
-        <v>12447</v>
+        <v>3892</v>
       </c>
       <c r="H191" s="138" t="n">
-        <v>1912</v>
+        <v>1098</v>
       </c>
       <c r="I191" s="138" t="n">
-        <v>10535</v>
+        <v>2794</v>
       </c>
       <c r="J191" s="139" t="n">
-        <v>379.49</v>
+        <v>119.74</v>
       </c>
       <c r="K191" s="139" t="n">
-        <v>398.33</v>
-      </c>
-      <c r="L191" s="235">
+        <v>119.39</v>
+      </c>
+      <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -19501,29 +19527,29 @@
       <c r="C192" s="140" t="n"/>
       <c r="D192" s="137" t="inlineStr">
         <is>
-          <t>光寶科(2301)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E192" s="138" t="n">
-        <v>323</v>
+        <v>12</v>
       </c>
       <c r="F192" s="138" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G192" s="138" t="n">
-        <v>7413</v>
+        <v>2749</v>
       </c>
       <c r="H192" s="138" t="n">
-        <v>77</v>
+        <v>1510</v>
       </c>
       <c r="I192" s="138" t="n">
-        <v>7336</v>
+        <v>1239</v>
       </c>
       <c r="J192" s="139" t="n">
-        <v>229.5</v>
+        <v>2291.08</v>
       </c>
       <c r="K192" s="139" t="n">
-        <v>257</v>
+        <v>2517</v>
       </c>
       <c r="L192" s="235">
         <f>F192*(K192-J192)</f>
@@ -19536,29 +19562,29 @@
       <c r="C193" s="140" t="n"/>
       <c r="D193" s="137" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>台達電(2308)</t>
         </is>
       </c>
       <c r="E193" s="138" t="n">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="F193" s="138" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="G193" s="138" t="n">
-        <v>3748</v>
+        <v>2672</v>
       </c>
       <c r="H193" s="138" t="n">
-        <v>1172</v>
+        <v>1617</v>
       </c>
       <c r="I193" s="138" t="n">
-        <v>2576</v>
+        <v>1055</v>
       </c>
       <c r="J193" s="139" t="n">
-        <v>430.8</v>
+        <v>1571.59</v>
       </c>
       <c r="K193" s="139" t="n">
-        <v>433.96</v>
+        <v>1617.3</v>
       </c>
       <c r="L193" s="235">
         <f>F193*(K193-J193)</f>
@@ -19571,31 +19597,31 @@
       <c r="C194" s="140" t="n"/>
       <c r="D194" s="137" t="inlineStr">
         <is>
-          <t>金像電(2368)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E194" s="138" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="F194" s="138" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="G194" s="138" t="n">
-        <v>3358</v>
+        <v>2445</v>
       </c>
       <c r="H194" s="138" t="n">
-        <v>87</v>
+        <v>1121</v>
       </c>
       <c r="I194" s="138" t="n">
-        <v>3271</v>
+        <v>1324</v>
       </c>
       <c r="J194" s="139" t="n">
-        <v>861</v>
+        <v>436.55</v>
       </c>
       <c r="K194" s="139" t="n">
-        <v>872</v>
-      </c>
-      <c r="L194" s="235">
+        <v>431.31</v>
+      </c>
+      <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -19606,29 +19632,29 @@
       <c r="C195" s="140" t="n"/>
       <c r="D195" s="137" t="inlineStr">
         <is>
-          <t>旺宏(2337)</t>
+          <t>穩懋(3105)</t>
         </is>
       </c>
       <c r="E195" s="138" t="n">
-        <v>238</v>
+        <v>76</v>
       </c>
       <c r="F195" s="138" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="G195" s="138" t="n">
-        <v>2574</v>
+        <v>2383</v>
       </c>
       <c r="H195" s="138" t="n">
-        <v>351</v>
+        <v>1576</v>
       </c>
       <c r="I195" s="138" t="n">
-        <v>2223</v>
+        <v>807</v>
       </c>
       <c r="J195" s="139" t="n">
-        <v>108.13</v>
+        <v>313.61</v>
       </c>
       <c r="K195" s="139" t="n">
-        <v>109.59</v>
+        <v>315.12</v>
       </c>
       <c r="L195" s="235">
         <f>F195*(K195-J195)</f>
@@ -19641,31 +19667,31 @@
       <c r="C196" s="140" t="n"/>
       <c r="D196" s="137" t="inlineStr">
         <is>
-          <t>亞翔(6139)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E196" s="138" t="n">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="F196" s="138" t="n">
-        <v>8</v>
+        <v>87</v>
       </c>
       <c r="G196" s="138" t="n">
-        <v>2266</v>
+        <v>1959</v>
       </c>
       <c r="H196" s="138" t="n">
-        <v>619</v>
+        <v>1466</v>
       </c>
       <c r="I196" s="138" t="n">
-        <v>1647</v>
+        <v>493</v>
       </c>
       <c r="J196" s="139" t="n">
-        <v>755.23</v>
+        <v>170.38</v>
       </c>
       <c r="K196" s="139" t="n">
-        <v>773.75</v>
-      </c>
-      <c r="L196" s="235">
+        <v>168.54</v>
+      </c>
+      <c r="L196" s="236">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -19676,29 +19702,29 @@
       <c r="C197" s="140" t="n"/>
       <c r="D197" s="137" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E197" s="138" t="n">
-        <v>191</v>
+        <v>430</v>
       </c>
       <c r="F197" s="138" t="n">
-        <v>64</v>
+        <v>275</v>
       </c>
       <c r="G197" s="138" t="n">
-        <v>2266</v>
+        <v>1939</v>
       </c>
       <c r="H197" s="138" t="n">
-        <v>771</v>
+        <v>1262</v>
       </c>
       <c r="I197" s="138" t="n">
-        <v>1495</v>
+        <v>677</v>
       </c>
       <c r="J197" s="139" t="n">
-        <v>118.62</v>
+        <v>45.09</v>
       </c>
       <c r="K197" s="139" t="n">
-        <v>120.5</v>
+        <v>45.9</v>
       </c>
       <c r="L197" s="235">
         <f>F197*(K197-J197)</f>
@@ -19711,29 +19737,29 @@
       <c r="C198" s="140" t="n"/>
       <c r="D198" s="137" t="inlineStr">
         <is>
-          <t>力積電(6770)</t>
+          <t>世芯-KY(3661)</t>
         </is>
       </c>
       <c r="E198" s="138" t="n">
-        <v>369</v>
+        <v>5</v>
       </c>
       <c r="F198" s="138" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G198" s="138" t="n">
-        <v>2023</v>
+        <v>1601</v>
       </c>
       <c r="H198" s="138" t="n">
-        <v>88</v>
+        <v>1290</v>
       </c>
       <c r="I198" s="138" t="n">
-        <v>1935</v>
+        <v>311</v>
       </c>
       <c r="J198" s="139" t="n">
-        <v>54.82</v>
+        <v>3201.2</v>
       </c>
       <c r="K198" s="139" t="n">
-        <v>55.19</v>
+        <v>3226.25</v>
       </c>
       <c r="L198" s="235">
         <f>F198*(K198-J198)</f>
@@ -19746,29 +19772,29 @@
       <c r="C199" s="140" t="n"/>
       <c r="D199" s="137" t="inlineStr">
         <is>
-          <t>文曄(3036)</t>
+          <t>台光電(2383)</t>
         </is>
       </c>
       <c r="E199" s="138" t="n">
-        <v>96</v>
+        <v>3</v>
       </c>
       <c r="F199" s="138" t="n">
         <v>1</v>
       </c>
       <c r="G199" s="138" t="n">
-        <v>1974</v>
+        <v>1572</v>
       </c>
       <c r="H199" s="138" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I199" s="138" t="n">
-        <v>1974</v>
+        <v>1552</v>
       </c>
       <c r="J199" s="139" t="n">
-        <v>205.66</v>
+        <v>5239</v>
       </c>
       <c r="K199" s="139" t="n">
-        <v>4</v>
+        <v>204</v>
       </c>
       <c r="L199" s="236">
         <f>F199*(K199-J199)</f>
@@ -30436,7 +30462,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="204" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-03 22:55 TW | 0/23 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-08-04 01:49 TW | 17/23 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-04 22:56
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -2273,8 +2273,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G28" s="248" t="n">
-        <v>0.1824037584120599</v>
+      <c r="G28" s="246" t="n">
+        <v>0.1827575179330782</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -30521,7 +30521,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-04 22:09 TW | 24/24 success | 來源: 富邦24/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-04 22:56 TW | 24/24 success | 來源: 富邦24/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-05 00:46
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="19">
+  <numFmts count="20">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -42,6 +42,7 @@
     <numFmt numFmtId="180" formatCode="0&quot; 檔 +78億 &quot;&quot;(昨10/5d9)&quot;"/>
     <numFmt numFmtId="181" formatCode="0.0%&quot; 市-1302億 &quot;&quot;(昨23/5d18)&quot;"/>
     <numFmt numFmtId="182" formatCode="0.0%&quot; 市-1297億 &quot;&quot;(昨23/5d18)&quot;"/>
+    <numFmt numFmtId="183" formatCode="0.0%&quot; 市-1301億 &quot;&quot;(昨23/5d18)&quot;"/>
   </numFmts>
   <fonts count="54">
     <font>
@@ -617,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="249">
+  <cellXfs count="250">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1195,6 +1196,9 @@
     <xf numFmtId="182" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="183" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2201,23 +2205,23 @@
         <v>10</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>293</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>陳律師</t>
         </is>
       </c>
-      <c r="H24" s="17" t="n">
+      <c r="J24" s="18" t="n">
         <v>272</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="J24" s="18" t="n">
-        <v>223</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2231,7 +2235,7 @@
         <v>7</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>1203</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -2256,7 +2260,7 @@
         </is>
       </c>
       <c r="G27" s="244" t="n">
-        <v>-90.55685</v>
+        <v>-89.31316</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
@@ -2273,8 +2277,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G28" s="246" t="n">
-        <v>0.1827575179330782</v>
+      <c r="G28" s="249" t="n">
+        <v>0.1832270153711584</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2385,11 +2389,11 @@
         </is>
       </c>
       <c r="D35" s="33" t="n">
-        <v>1407222</v>
+        <v>1423998</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.6%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2421,7 +2425,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.7%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -3063,7 +3067,7 @@
         </is>
       </c>
       <c r="C66" s="33" t="n">
-        <v>1370793</v>
+        <v>1385934</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3079,7 +3083,7 @@
         </is>
       </c>
       <c r="G66" s="33" t="n">
-        <v>110105</v>
+        <v>118606</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -3090,7 +3094,7 @@
         <v>97103</v>
       </c>
       <c r="J66" s="214" t="n">
-        <v>0.3376421531186692</v>
+        <v>0.3400869954532483</v>
       </c>
     </row>
     <row r="67">
@@ -5000,7 +5004,7 @@
     <row r="33" ht="22" customHeight="1">
       <c r="C33" s="247" t="inlineStr">
         <is>
-          <t>-91 億 淨買</t>
+          <t>-89 億 淨買</t>
         </is>
       </c>
     </row>
@@ -19544,7 +19548,7 @@
         </is>
       </c>
       <c r="E191" s="138" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F191" s="138" t="n">
         <v>1</v>
@@ -19559,7 +19563,7 @@
         <v>12434</v>
       </c>
       <c r="J191" s="139" t="n">
-        <v>1019.34</v>
+        <v>1027.77</v>
       </c>
       <c r="K191" s="139" t="n">
         <v>25</v>
@@ -19614,10 +19618,10 @@
         </is>
       </c>
       <c r="E193" s="138" t="n">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="F193" s="138" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G193" s="138" t="n">
         <v>10447</v>
@@ -19629,12 +19633,12 @@
         <v>4615</v>
       </c>
       <c r="J193" s="139" t="n">
-        <v>414.58</v>
+        <v>435.31</v>
       </c>
       <c r="K193" s="139" t="n">
-        <v>428.85</v>
-      </c>
-      <c r="L193" s="235">
+        <v>435.25</v>
+      </c>
+      <c r="L193" s="236">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -19645,31 +19649,31 @@
       <c r="C194" s="140" t="n"/>
       <c r="D194" s="137" t="inlineStr">
         <is>
-          <t>貿聯-KY(3665)</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E194" s="138" t="n">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="F194" s="138" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="G194" s="138" t="n">
-        <v>4752</v>
+        <v>8501</v>
       </c>
       <c r="H194" s="138" t="n">
-        <v>54</v>
+        <v>3049</v>
       </c>
       <c r="I194" s="138" t="n">
-        <v>4698</v>
+        <v>5452</v>
       </c>
       <c r="J194" s="139" t="n">
-        <v>2263.1</v>
+        <v>924</v>
       </c>
       <c r="K194" s="139" t="n">
-        <v>538</v>
-      </c>
-      <c r="L194" s="236">
+        <v>924</v>
+      </c>
+      <c r="L194" s="235">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -19680,29 +19684,29 @@
       <c r="C195" s="140" t="n"/>
       <c r="D195" s="137" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>貿聯-KY(3665)</t>
         </is>
       </c>
       <c r="E195" s="138" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="F195" s="138" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="G195" s="138" t="n">
-        <v>3676</v>
+        <v>4752</v>
       </c>
       <c r="H195" s="138" t="n">
-        <v>2996</v>
+        <v>54</v>
       </c>
       <c r="I195" s="138" t="n">
-        <v>680</v>
+        <v>4698</v>
       </c>
       <c r="J195" s="139" t="n">
-        <v>565.5700000000001</v>
+        <v>2263.1</v>
       </c>
       <c r="K195" s="139" t="n">
-        <v>565.1900000000001</v>
+        <v>538</v>
       </c>
       <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
@@ -19715,31 +19719,31 @@
       <c r="C196" s="140" t="n"/>
       <c r="D196" s="137" t="inlineStr">
         <is>
-          <t>日月光投控(3711)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E196" s="138" t="n">
-        <v>48</v>
+        <v>138</v>
       </c>
       <c r="F196" s="138" t="n">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="G196" s="138" t="n">
-        <v>2813</v>
+        <v>3676</v>
       </c>
       <c r="H196" s="138" t="n">
-        <v>233</v>
+        <v>2996</v>
       </c>
       <c r="I196" s="138" t="n">
-        <v>2580</v>
+        <v>680</v>
       </c>
       <c r="J196" s="139" t="n">
-        <v>585.98</v>
+        <v>266.39</v>
       </c>
       <c r="K196" s="139" t="n">
-        <v>582</v>
-      </c>
-      <c r="L196" s="236">
+        <v>507.71</v>
+      </c>
+      <c r="L196" s="235">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -19750,29 +19754,29 @@
       <c r="C197" s="140" t="n"/>
       <c r="D197" s="137" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E197" s="138" t="n">
-        <v>141</v>
+        <v>244</v>
       </c>
       <c r="F197" s="138" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="G197" s="138" t="n">
-        <v>2410</v>
+        <v>2891</v>
       </c>
       <c r="H197" s="138" t="n">
-        <v>1457</v>
+        <v>557</v>
       </c>
       <c r="I197" s="138" t="n">
-        <v>953</v>
+        <v>2334</v>
       </c>
       <c r="J197" s="139" t="n">
-        <v>170.89</v>
+        <v>118.5</v>
       </c>
       <c r="K197" s="139" t="n">
-        <v>171.36</v>
+        <v>118.51</v>
       </c>
       <c r="L197" s="235">
         <f>F197*(K197-J197)</f>
@@ -19785,31 +19789,31 @@
       <c r="C198" s="140" t="n"/>
       <c r="D198" s="137" t="inlineStr">
         <is>
-          <t>勤誠(8210)</t>
+          <t>日月光投控(3711)</t>
         </is>
       </c>
       <c r="E198" s="138" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="F198" s="138" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G198" s="138" t="n">
-        <v>2256</v>
+        <v>2813</v>
       </c>
       <c r="H198" s="138" t="n">
-        <v>574</v>
+        <v>233</v>
       </c>
       <c r="I198" s="138" t="n">
-        <v>1682</v>
+        <v>2580</v>
       </c>
       <c r="J198" s="139" t="n">
-        <v>1127.9</v>
+        <v>585.98</v>
       </c>
       <c r="K198" s="139" t="n">
-        <v>1147.4</v>
-      </c>
-      <c r="L198" s="235">
+        <v>582</v>
+      </c>
+      <c r="L198" s="236">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -30521,7 +30525,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 00:02 TW | 24/24 success | 來源: 富邦24/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 00:46 TW | 24/24 success | 來源: 富邦24/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-05 01:43
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="20">
+  <numFmts count="21">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -43,6 +43,7 @@
     <numFmt numFmtId="181" formatCode="0.0%&quot; 市-1302億 &quot;&quot;(昨23/5d18)&quot;"/>
     <numFmt numFmtId="182" formatCode="0.0%&quot; 市-1297億 &quot;&quot;(昨23/5d18)&quot;"/>
     <numFmt numFmtId="183" formatCode="0.0%&quot; 市-1301億 &quot;&quot;(昨23/5d18)&quot;"/>
+    <numFmt numFmtId="184" formatCode="0.0%&quot; 市-1295億 &quot;&quot;(昨23/5d18)&quot;"/>
   </numFmts>
   <fonts count="54">
     <font>
@@ -618,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="250">
+  <cellXfs count="251">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1199,6 +1200,9 @@
     <xf numFmtId="183" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="184" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2260,7 +2264,7 @@
         </is>
       </c>
       <c r="G27" s="244" t="n">
-        <v>-89.31316</v>
+        <v>-89.41092999999999</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
@@ -2277,8 +2281,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G28" s="249" t="n">
-        <v>0.1832270153711584</v>
+      <c r="G28" s="250" t="n">
+        <v>0.1827521554957778</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2357,7 +2361,7 @@
         </is>
       </c>
       <c r="D34" s="33" t="n">
-        <v>1453099</v>
+        <v>1452482</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2389,7 +2393,7 @@
         </is>
       </c>
       <c r="D35" s="33" t="n">
-        <v>1423998</v>
+        <v>1423818</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -3067,7 +3071,7 @@
         </is>
       </c>
       <c r="C66" s="33" t="n">
-        <v>1385934</v>
+        <v>1385755</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3094,7 +3098,7 @@
         <v>97103</v>
       </c>
       <c r="J66" s="214" t="n">
-        <v>0.3400869954532483</v>
+        <v>0.3401311213304923</v>
       </c>
     </row>
     <row r="67">
@@ -3104,7 +3108,7 @@
         </is>
       </c>
       <c r="C67" s="33" t="n">
-        <v>1231906</v>
+        <v>1231370</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3131,7 +3135,7 @@
         <v>69680</v>
       </c>
       <c r="J67" s="214" t="n">
-        <v>0.2423758990033248</v>
+        <v>0.2424814416011698</v>
       </c>
     </row>
     <row r="68">
@@ -3474,7 +3478,7 @@
         </is>
       </c>
       <c r="C77" s="33" t="n">
-        <v>38408</v>
+        <v>38131</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3501,7 +3505,7 @@
         <v>3386</v>
       </c>
       <c r="J77" s="214" t="n">
-        <v>0.3562154210656495</v>
+        <v>0.3588040302742622</v>
       </c>
     </row>
     <row r="78">
@@ -28128,33 +28132,33 @@
       <c r="A417" s="187" t="n"/>
       <c r="B417" s="187" t="n"/>
       <c r="C417" s="187" t="n"/>
-      <c r="D417" s="240" t="inlineStr">
-        <is>
-          <t>明遠精密(7704)</t>
-        </is>
-      </c>
-      <c r="E417" s="241" t="n">
-        <v>58</v>
-      </c>
-      <c r="F417" s="241" t="n">
+      <c r="D417" s="184" t="inlineStr">
+        <is>
+          <t>合晶(6182)</t>
+        </is>
+      </c>
+      <c r="E417" s="185" t="n">
+        <v>31</v>
+      </c>
+      <c r="F417" s="185" t="n">
+        <v>1</v>
+      </c>
+      <c r="G417" s="185" t="n">
+        <v>296</v>
+      </c>
+      <c r="H417" s="185" t="n">
         <v>0</v>
       </c>
-      <c r="G417" s="241" t="n">
-        <v>353</v>
-      </c>
-      <c r="H417" s="241" t="n">
-        <v>0</v>
-      </c>
-      <c r="I417" s="241" t="n">
-        <v>353</v>
-      </c>
-      <c r="J417" s="242" t="n">
-        <v>60.9</v>
-      </c>
-      <c r="K417" s="242" t="n">
-        <v>0</v>
-      </c>
-      <c r="L417" s="243">
+      <c r="I417" s="185" t="n">
+        <v>296</v>
+      </c>
+      <c r="J417" s="186" t="n">
+        <v>95.52</v>
+      </c>
+      <c r="K417" s="186" t="n">
+        <v>5</v>
+      </c>
+      <c r="L417" s="236">
         <f>F417*(K417-J417)</f>
         <v/>
       </c>
@@ -28165,31 +28169,31 @@
       <c r="C418" s="187" t="n"/>
       <c r="D418" s="184" t="inlineStr">
         <is>
-          <t>合晶(6182)</t>
+          <t>閎康(3587)</t>
         </is>
       </c>
       <c r="E418" s="185" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F418" s="185" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G418" s="185" t="n">
-        <v>296</v>
+        <v>252</v>
       </c>
       <c r="H418" s="185" t="n">
         <v>0</v>
       </c>
       <c r="I418" s="185" t="n">
-        <v>296</v>
+        <v>252</v>
       </c>
       <c r="J418" s="186" t="n">
-        <v>95.52</v>
+        <v>251.5</v>
       </c>
       <c r="K418" s="186" t="n">
-        <v>5</v>
-      </c>
-      <c r="L418" s="236">
+        <v>0</v>
+      </c>
+      <c r="L418" s="235">
         <f>F418*(K418-J418)</f>
         <v/>
       </c>
@@ -30525,7 +30529,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 00:46 TW | 24/24 success | 來源: 富邦24/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 01:43 TW | 23/23 success | 來源: 富邦23/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-05 22:57
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="G30" s="251" t="n">
-        <v>-187.38063</v>
+        <v>-187.36154</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="G31" s="253" t="n">
-        <v>0.1593232770364576</v>
+        <v>0.1593540390485123</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>380258</v>
+        <v>380239</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         </is>
       </c>
       <c r="D41" s="33" t="n">
-        <v>375000</v>
+        <v>374969</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>蔣承翰</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>陳律師 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>蔣承翰 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>5 檔</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
-          <t>蔣承翰</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D49" s="41" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="E49" s="41" t="inlineStr">
         <is>
-          <t>蔣承翰 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" s="41" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2854,12 +2854,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>強森 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>4 檔</t>
+          <t>3 檔</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2881,12 +2881,12 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
         <is>
-          <t>4 檔</t>
+          <t>3 檔</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2908,12 +2908,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>4 檔</t>
+          <t>3 檔</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C53" s="41" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D53" s="41" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="41" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>張濬安(航海王)</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3329,7 +3329,7 @@
         </is>
       </c>
       <c r="C70" s="33" t="n">
-        <v>310124</v>
+        <v>310105</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3356,7 +3356,7 @@
         <v>16869</v>
       </c>
       <c r="J70" s="214" t="n">
-        <v>0.2019043344261217</v>
+        <v>0.2019167701262476</v>
       </c>
     </row>
     <row r="71">
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="C71" s="33" t="n">
-        <v>280810</v>
+        <v>280769</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3393,7 +3393,7 @@
         <v>20725</v>
       </c>
       <c r="J71" s="214" t="n">
-        <v>0.3446970277002737</v>
+        <v>0.344746749106917</v>
       </c>
     </row>
     <row r="72">
@@ -28263,31 +28263,31 @@
       <c r="C417" s="187" t="n"/>
       <c r="D417" s="240" t="inlineStr">
         <is>
-          <t>亞泰金屬(6727)</t>
+          <t>前鼎(4908)</t>
         </is>
       </c>
       <c r="E417" s="241" t="n">
-        <v>104</v>
+        <v>164</v>
       </c>
       <c r="F417" s="241" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G417" s="241" t="n">
-        <v>4233</v>
+        <v>2714</v>
       </c>
       <c r="H417" s="241" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I417" s="241" t="n">
-        <v>4224</v>
+        <v>2714</v>
       </c>
       <c r="J417" s="242" t="n">
-        <v>406.98</v>
+        <v>165.5</v>
       </c>
       <c r="K417" s="242" t="n">
-        <v>88</v>
-      </c>
-      <c r="L417" s="255">
+        <v>0</v>
+      </c>
+      <c r="L417" s="243">
         <f>F417*(K417-J417)</f>
         <v/>
       </c>
@@ -28296,33 +28296,33 @@
       <c r="A418" s="187" t="n"/>
       <c r="B418" s="187" t="n"/>
       <c r="C418" s="187" t="n"/>
-      <c r="D418" s="240" t="inlineStr">
-        <is>
-          <t>前鼎(4908)</t>
-        </is>
-      </c>
-      <c r="E418" s="241" t="n">
-        <v>164</v>
-      </c>
-      <c r="F418" s="241" t="n">
-        <v>0</v>
-      </c>
-      <c r="G418" s="241" t="n">
-        <v>2714</v>
-      </c>
-      <c r="H418" s="241" t="n">
-        <v>0</v>
-      </c>
-      <c r="I418" s="241" t="n">
-        <v>2714</v>
-      </c>
-      <c r="J418" s="242" t="n">
-        <v>165.5</v>
-      </c>
-      <c r="K418" s="242" t="n">
-        <v>0</v>
-      </c>
-      <c r="L418" s="243">
+      <c r="D418" s="184" t="inlineStr">
+        <is>
+          <t>聯亞(3081)</t>
+        </is>
+      </c>
+      <c r="E418" s="185" t="n">
+        <v>10</v>
+      </c>
+      <c r="F418" s="185" t="n">
+        <v>1</v>
+      </c>
+      <c r="G418" s="185" t="n">
+        <v>2168</v>
+      </c>
+      <c r="H418" s="185" t="n">
+        <v>231</v>
+      </c>
+      <c r="I418" s="185" t="n">
+        <v>1937</v>
+      </c>
+      <c r="J418" s="186" t="n">
+        <v>2167.6</v>
+      </c>
+      <c r="K418" s="186" t="n">
+        <v>2309</v>
+      </c>
+      <c r="L418" s="235">
         <f>F418*(K418-J418)</f>
         <v/>
       </c>
@@ -30574,7 +30574,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 21:40 TW | 19/19 success | 來源: 富邦19/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 22:57 TW | 18/18 success | 來源: 富邦18/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-05 23:55
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="G30" s="251" t="n">
-        <v>-187.36154</v>
+        <v>-187.38063</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="G31" s="253" t="n">
-        <v>0.1593540390485123</v>
+        <v>0.1590669231384998</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>380239</v>
+        <v>380258</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         </is>
       </c>
       <c r="D41" s="33" t="n">
-        <v>374969</v>
+        <v>375000</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>蔣承翰</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>蔣承翰 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>5 檔</t>
+          <t>6 檔</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>蔣承翰</t>
         </is>
       </c>
       <c r="D49" s="41" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="E49" s="41" t="inlineStr">
         <is>
-          <t>陳律師 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>蔣承翰 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" s="41" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2854,12 +2854,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>3 檔</t>
+          <t>4 檔</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王)</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2881,12 +2881,12 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
         <is>
-          <t>3 檔</t>
+          <t>4 檔</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2908,12 +2908,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>強森 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>3 檔</t>
+          <t>4 檔</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C53" s="41" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D53" s="41" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="41" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3329,7 +3329,7 @@
         </is>
       </c>
       <c r="C70" s="33" t="n">
-        <v>310105</v>
+        <v>310124</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3356,7 +3356,7 @@
         <v>16869</v>
       </c>
       <c r="J70" s="214" t="n">
-        <v>0.2019167701262476</v>
+        <v>0.2019043344261217</v>
       </c>
     </row>
     <row r="71">
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="C71" s="33" t="n">
-        <v>280769</v>
+        <v>280810</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3393,7 +3393,7 @@
         <v>20725</v>
       </c>
       <c r="J71" s="214" t="n">
-        <v>0.344746749106917</v>
+        <v>0.3446970277002737</v>
       </c>
     </row>
     <row r="72">
@@ -28263,31 +28263,31 @@
       <c r="C417" s="187" t="n"/>
       <c r="D417" s="240" t="inlineStr">
         <is>
-          <t>前鼎(4908)</t>
+          <t>亞泰金屬(6727)</t>
         </is>
       </c>
       <c r="E417" s="241" t="n">
-        <v>164</v>
+        <v>104</v>
       </c>
       <c r="F417" s="241" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G417" s="241" t="n">
-        <v>2714</v>
+        <v>4233</v>
       </c>
       <c r="H417" s="241" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I417" s="241" t="n">
-        <v>2714</v>
+        <v>4224</v>
       </c>
       <c r="J417" s="242" t="n">
-        <v>165.5</v>
+        <v>406.98</v>
       </c>
       <c r="K417" s="242" t="n">
-        <v>0</v>
-      </c>
-      <c r="L417" s="243">
+        <v>88</v>
+      </c>
+      <c r="L417" s="255">
         <f>F417*(K417-J417)</f>
         <v/>
       </c>
@@ -28296,33 +28296,33 @@
       <c r="A418" s="187" t="n"/>
       <c r="B418" s="187" t="n"/>
       <c r="C418" s="187" t="n"/>
-      <c r="D418" s="184" t="inlineStr">
-        <is>
-          <t>聯亞(3081)</t>
-        </is>
-      </c>
-      <c r="E418" s="185" t="n">
-        <v>10</v>
-      </c>
-      <c r="F418" s="185" t="n">
-        <v>1</v>
-      </c>
-      <c r="G418" s="185" t="n">
-        <v>2168</v>
-      </c>
-      <c r="H418" s="185" t="n">
-        <v>231</v>
-      </c>
-      <c r="I418" s="185" t="n">
-        <v>1937</v>
-      </c>
-      <c r="J418" s="186" t="n">
-        <v>2167.6</v>
-      </c>
-      <c r="K418" s="186" t="n">
-        <v>2309</v>
-      </c>
-      <c r="L418" s="235">
+      <c r="D418" s="240" t="inlineStr">
+        <is>
+          <t>前鼎(4908)</t>
+        </is>
+      </c>
+      <c r="E418" s="241" t="n">
+        <v>164</v>
+      </c>
+      <c r="F418" s="241" t="n">
+        <v>0</v>
+      </c>
+      <c r="G418" s="241" t="n">
+        <v>2714</v>
+      </c>
+      <c r="H418" s="241" t="n">
+        <v>0</v>
+      </c>
+      <c r="I418" s="241" t="n">
+        <v>2714</v>
+      </c>
+      <c r="J418" s="242" t="n">
+        <v>165.5</v>
+      </c>
+      <c r="K418" s="242" t="n">
+        <v>0</v>
+      </c>
+      <c r="L418" s="243">
         <f>F418*(K418-J418)</f>
         <v/>
       </c>
@@ -30574,7 +30574,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 22:57 TW | 18/18 success | 來源: 富邦18/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 23:55 TW | 19/19 success | 來源: 富邦19/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-06 00:38
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="24">
+  <numFmts count="25">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-64/5d-140)&quot;;-0&quot; 億 (昨-64/5d-140)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +122億 &quot;&quot;(昨5/5d9)&quot;"/>
@@ -48,6 +48,7 @@
     <numFmt numFmtId="185" formatCode="+0&quot; 億 (昨-89/5d-59)&quot;;-0&quot; 億 (昨-89/5d-59)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="186" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨9/5d8)&quot;"/>
     <numFmt numFmtId="187" formatCode="0.0%&quot; 市-478億 &quot;&quot;(昨18/5d18)&quot;"/>
+    <numFmt numFmtId="188" formatCode="0.0%&quot; 市-475億 &quot;&quot;(昨18/5d18)&quot;"/>
   </numFmts>
   <fonts count="54">
     <font>
@@ -623,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="256">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1220,6 +1221,9 @@
     <xf numFmtId="176" fontId="5" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="188" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1305,12 +1309,12 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 60.9%
+領頭大戶「張濬安(航海王)」獨佔比 60.3%
   • 領頭金額 136,742 萬
-  • 合計淨買 224,645 萬
+  • 合計淨買 226,692 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 61%,
+實質 1 人下注佔 60%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1831,7 +1835,7 @@
         <v>10</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
@@ -1847,7 +1851,7 @@
         </is>
       </c>
       <c r="J16" s="18" t="n">
-        <v>56060</v>
+        <v>58107</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1861,7 +1865,7 @@
         <v>7</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>224645</v>
+        <v>226692</v>
       </c>
     </row>
     <row r="17">
@@ -2239,7 +2243,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
@@ -2247,7 +2251,7 @@
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>5060</v>
+        <v>4888</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2269,7 +2273,7 @@
         <v>8</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>19002</v>
+        <v>18830</v>
       </c>
     </row>
     <row r="25">
@@ -2392,7 +2396,7 @@
         <v>10</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
@@ -2422,7 +2426,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>7730</v>
+        <v>7848</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2447,7 +2451,7 @@
         </is>
       </c>
       <c r="G30" s="251" t="n">
-        <v>-187.38063</v>
+        <v>-183.99805</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2464,8 +2468,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="253" t="n">
-        <v>0.1590669231384998</v>
+      <c r="G31" s="256" t="n">
+        <v>0.1595358900128013</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2548,7 +2552,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>35.6%</t>
+          <t>35.5%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2576,11 +2580,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1489607</v>
+        <v>1509116</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2592,7 +2596,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>224645</v>
+        <v>226692</v>
       </c>
       <c r="I38" s="213" t="n">
         <v>0.0206</v>
@@ -2844,22 +2848,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>強森 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>4 檔</t>
+          <t>5 檔</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2875,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2881,7 +2885,7 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
@@ -2898,7 +2902,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2908,7 +2912,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3218,7 +3222,7 @@
         </is>
       </c>
       <c r="C67" s="33" t="n">
-        <v>1371660</v>
+        <v>1389992</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3245,7 +3249,7 @@
         <v>124487</v>
       </c>
       <c r="J67" s="214" t="n">
-        <v>0.3274504853571938</v>
+        <v>0.3231317667636168</v>
       </c>
     </row>
     <row r="68">
@@ -5137,7 +5141,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="247" t="inlineStr">
         <is>
-          <t>-187 億 淨買</t>
+          <t>-184 億 淨買</t>
         </is>
       </c>
     </row>
@@ -19642,31 +19646,31 @@
       <c r="C190" s="140" t="n"/>
       <c r="D190" s="137" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E190" s="138" t="n">
-        <v>696</v>
+        <v>752</v>
       </c>
       <c r="F190" s="138" t="n">
-        <v>133</v>
+        <v>726</v>
       </c>
       <c r="G190" s="138" t="n">
-        <v>8692</v>
+        <v>13310</v>
       </c>
       <c r="H190" s="138" t="n">
-        <v>1658</v>
+        <v>12850</v>
       </c>
       <c r="I190" s="138" t="n">
-        <v>7034</v>
+        <v>460</v>
       </c>
       <c r="J190" s="139" t="n">
-        <v>124.89</v>
+        <v>177</v>
       </c>
       <c r="K190" s="139" t="n">
-        <v>124.67</v>
-      </c>
-      <c r="L190" s="236">
+        <v>177</v>
+      </c>
+      <c r="L190" s="235">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -19677,31 +19681,31 @@
       <c r="C191" s="140" t="n"/>
       <c r="D191" s="137" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E191" s="138" t="n">
-        <v>79</v>
+        <v>712</v>
       </c>
       <c r="F191" s="138" t="n">
-        <v>34</v>
+        <v>136</v>
       </c>
       <c r="G191" s="138" t="n">
-        <v>8310</v>
+        <v>8692</v>
       </c>
       <c r="H191" s="138" t="n">
-        <v>3634</v>
+        <v>1658</v>
       </c>
       <c r="I191" s="138" t="n">
-        <v>4676</v>
+        <v>7034</v>
       </c>
       <c r="J191" s="139" t="n">
-        <v>1051.9</v>
+        <v>122.08</v>
       </c>
       <c r="K191" s="139" t="n">
-        <v>1068.76</v>
-      </c>
-      <c r="L191" s="235">
+        <v>121.92</v>
+      </c>
+      <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -19712,29 +19716,29 @@
       <c r="C192" s="140" t="n"/>
       <c r="D192" s="137" t="inlineStr">
         <is>
-          <t>文曄(3036)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E192" s="138" t="n">
-        <v>352</v>
+        <v>80</v>
       </c>
       <c r="F192" s="138" t="n">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="G192" s="138" t="n">
-        <v>7916</v>
+        <v>8310</v>
       </c>
       <c r="H192" s="138" t="n">
-        <v>1500</v>
+        <v>3634</v>
       </c>
       <c r="I192" s="138" t="n">
-        <v>6416</v>
+        <v>4676</v>
       </c>
       <c r="J192" s="139" t="n">
-        <v>224.89</v>
+        <v>1038.75</v>
       </c>
       <c r="K192" s="139" t="n">
-        <v>220.56</v>
+        <v>1038.23</v>
       </c>
       <c r="L192" s="236">
         <f>F192*(K192-J192)</f>
@@ -19747,31 +19751,31 @@
       <c r="C193" s="140" t="n"/>
       <c r="D193" s="137" t="inlineStr">
         <is>
-          <t>旺宏(2337)</t>
+          <t>文曄(3036)</t>
         </is>
       </c>
       <c r="E193" s="138" t="n">
-        <v>500</v>
+        <v>352</v>
       </c>
       <c r="F193" s="138" t="n">
-        <v>259</v>
+        <v>67</v>
       </c>
       <c r="G193" s="138" t="n">
-        <v>6135</v>
+        <v>7916</v>
       </c>
       <c r="H193" s="138" t="n">
-        <v>3188</v>
+        <v>1500</v>
       </c>
       <c r="I193" s="138" t="n">
-        <v>2947</v>
+        <v>6416</v>
       </c>
       <c r="J193" s="139" t="n">
-        <v>122.71</v>
+        <v>224.89</v>
       </c>
       <c r="K193" s="139" t="n">
-        <v>123.09</v>
-      </c>
-      <c r="L193" s="235">
+        <v>223.85</v>
+      </c>
+      <c r="L193" s="236">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -19782,29 +19786,29 @@
       <c r="C194" s="140" t="n"/>
       <c r="D194" s="137" t="inlineStr">
         <is>
-          <t>強茂(2481)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E194" s="138" t="n">
-        <v>332</v>
+        <v>130</v>
       </c>
       <c r="F194" s="138" t="n">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="G194" s="138" t="n">
-        <v>4589</v>
+        <v>6135</v>
       </c>
       <c r="H194" s="138" t="n">
-        <v>245</v>
+        <v>3188</v>
       </c>
       <c r="I194" s="138" t="n">
-        <v>4344</v>
+        <v>2947</v>
       </c>
       <c r="J194" s="139" t="n">
-        <v>138.22</v>
+        <v>471.95</v>
       </c>
       <c r="K194" s="139" t="n">
-        <v>136.33</v>
+        <v>419.49</v>
       </c>
       <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
@@ -19817,29 +19821,29 @@
       <c r="C195" s="140" t="n"/>
       <c r="D195" s="137" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>強茂(2481)</t>
         </is>
       </c>
       <c r="E195" s="138" t="n">
-        <v>185</v>
+        <v>342</v>
       </c>
       <c r="F195" s="138" t="n">
-        <v>164</v>
+        <v>18</v>
       </c>
       <c r="G195" s="138" t="n">
-        <v>3120</v>
+        <v>4589</v>
       </c>
       <c r="H195" s="138" t="n">
-        <v>2775</v>
+        <v>245</v>
       </c>
       <c r="I195" s="138" t="n">
-        <v>345</v>
+        <v>4344</v>
       </c>
       <c r="J195" s="139" t="n">
-        <v>168.64</v>
+        <v>134.18</v>
       </c>
       <c r="K195" s="139" t="n">
-        <v>169.2</v>
+        <v>136.33</v>
       </c>
       <c r="L195" s="235">
         <f>F195*(K195-J195)</f>
@@ -19852,29 +19856,29 @@
       <c r="C196" s="140" t="n"/>
       <c r="D196" s="137" t="inlineStr">
         <is>
-          <t>環球晶(6488)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E196" s="138" t="n">
-        <v>27</v>
+        <v>101</v>
       </c>
       <c r="F196" s="138" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="G196" s="138" t="n">
-        <v>2363</v>
+        <v>4494</v>
       </c>
       <c r="H196" s="138" t="n">
-        <v>1169</v>
+        <v>2448</v>
       </c>
       <c r="I196" s="138" t="n">
-        <v>1194</v>
+        <v>2046</v>
       </c>
       <c r="J196" s="139" t="n">
-        <v>875.22</v>
+        <v>445</v>
       </c>
       <c r="K196" s="139" t="n">
-        <v>899.38</v>
+        <v>445</v>
       </c>
       <c r="L196" s="235">
         <f>F196*(K196-J196)</f>
@@ -19887,29 +19891,29 @@
       <c r="C197" s="140" t="n"/>
       <c r="D197" s="137" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E197" s="138" t="n">
-        <v>403</v>
+        <v>185</v>
       </c>
       <c r="F197" s="138" t="n">
-        <v>367</v>
+        <v>164</v>
       </c>
       <c r="G197" s="138" t="n">
-        <v>1926</v>
+        <v>3120</v>
       </c>
       <c r="H197" s="138" t="n">
-        <v>1754</v>
+        <v>2775</v>
       </c>
       <c r="I197" s="138" t="n">
-        <v>172</v>
+        <v>345</v>
       </c>
       <c r="J197" s="139" t="n">
-        <v>47.8</v>
+        <v>168.64</v>
       </c>
       <c r="K197" s="139" t="n">
-        <v>47.8</v>
+        <v>169.2</v>
       </c>
       <c r="L197" s="235">
         <f>F197*(K197-J197)</f>
@@ -19922,29 +19926,29 @@
       <c r="C198" s="140" t="n"/>
       <c r="D198" s="137" t="inlineStr">
         <is>
-          <t>力成(6239)</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E198" s="138" t="n">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="F198" s="138" t="n">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="G198" s="138" t="n">
-        <v>1909</v>
+        <v>2363</v>
       </c>
       <c r="H198" s="138" t="n">
-        <v>1678</v>
+        <v>1169</v>
       </c>
       <c r="I198" s="138" t="n">
-        <v>231</v>
+        <v>1194</v>
       </c>
       <c r="J198" s="139" t="n">
-        <v>258</v>
+        <v>875.22</v>
       </c>
       <c r="K198" s="139" t="n">
-        <v>258.12</v>
+        <v>899.38</v>
       </c>
       <c r="L198" s="235">
         <f>F198*(K198-J198)</f>
@@ -30574,7 +30578,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-05 23:55 TW | 19/19 success | 來源: 富邦19/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-06 00:38 TW | 19/19 success | 來源: 富邦19/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-06 01:29
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -1309,12 +1309,12 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 60.3%
+領頭大戶「張濬安(航海王)」獨佔比 60.9%
   • 領頭金額 136,742 萬
-  • 合計淨買 226,692 萬
+  • 合計淨買 224,645 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 60%,
+實質 1 人下注佔 61%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1835,7 +1835,7 @@
         <v>10</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="J16" s="18" t="n">
-        <v>58107</v>
+        <v>56060</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         <v>7</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>226692</v>
+        <v>224645</v>
       </c>
     </row>
     <row r="17">
@@ -2243,7 +2243,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>4888</v>
+        <v>5060</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>8</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>18830</v>
+        <v>19002</v>
       </c>
     </row>
     <row r="25">
@@ -2396,7 +2396,7 @@
         <v>10</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
@@ -2426,7 +2426,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>7848</v>
+        <v>7730</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="G30" s="251" t="n">
-        <v>-183.99805</v>
+        <v>-187.38063</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2468,8 +2468,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="256" t="n">
-        <v>0.1595358900128013</v>
+      <c r="G31" s="253" t="n">
+        <v>0.1590669231384998</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>35.6%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2580,11 +2580,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1509116</v>
+        <v>1489607</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>226692</v>
+        <v>224645</v>
       </c>
       <c r="I38" s="213" t="n">
         <v>0.0206</v>
@@ -2848,22 +2848,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>5 檔</t>
+          <t>4 檔</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>強森 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3222,7 +3222,7 @@
         </is>
       </c>
       <c r="C67" s="33" t="n">
-        <v>1389992</v>
+        <v>1371660</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3249,7 +3249,7 @@
         <v>124487</v>
       </c>
       <c r="J67" s="214" t="n">
-        <v>0.3231317667636168</v>
+        <v>0.3274504853571938</v>
       </c>
     </row>
     <row r="68">
@@ -5141,7 +5141,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="247" t="inlineStr">
         <is>
-          <t>-184 億 淨買</t>
+          <t>-187 億 淨買</t>
         </is>
       </c>
     </row>
@@ -19646,31 +19646,31 @@
       <c r="C190" s="140" t="n"/>
       <c r="D190" s="137" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E190" s="138" t="n">
-        <v>752</v>
+        <v>696</v>
       </c>
       <c r="F190" s="138" t="n">
-        <v>726</v>
+        <v>133</v>
       </c>
       <c r="G190" s="138" t="n">
-        <v>13310</v>
+        <v>8692</v>
       </c>
       <c r="H190" s="138" t="n">
-        <v>12850</v>
+        <v>1658</v>
       </c>
       <c r="I190" s="138" t="n">
-        <v>460</v>
+        <v>7034</v>
       </c>
       <c r="J190" s="139" t="n">
-        <v>177</v>
+        <v>124.89</v>
       </c>
       <c r="K190" s="139" t="n">
-        <v>177</v>
-      </c>
-      <c r="L190" s="235">
+        <v>124.67</v>
+      </c>
+      <c r="L190" s="236">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -19681,31 +19681,31 @@
       <c r="C191" s="140" t="n"/>
       <c r="D191" s="137" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E191" s="138" t="n">
-        <v>712</v>
+        <v>79</v>
       </c>
       <c r="F191" s="138" t="n">
-        <v>136</v>
+        <v>34</v>
       </c>
       <c r="G191" s="138" t="n">
-        <v>8692</v>
+        <v>8310</v>
       </c>
       <c r="H191" s="138" t="n">
-        <v>1658</v>
+        <v>3634</v>
       </c>
       <c r="I191" s="138" t="n">
-        <v>7034</v>
+        <v>4676</v>
       </c>
       <c r="J191" s="139" t="n">
-        <v>122.08</v>
+        <v>1051.9</v>
       </c>
       <c r="K191" s="139" t="n">
-        <v>121.92</v>
-      </c>
-      <c r="L191" s="236">
+        <v>1068.76</v>
+      </c>
+      <c r="L191" s="235">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -19716,29 +19716,29 @@
       <c r="C192" s="140" t="n"/>
       <c r="D192" s="137" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>文曄(3036)</t>
         </is>
       </c>
       <c r="E192" s="138" t="n">
-        <v>80</v>
+        <v>352</v>
       </c>
       <c r="F192" s="138" t="n">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="G192" s="138" t="n">
-        <v>8310</v>
+        <v>7916</v>
       </c>
       <c r="H192" s="138" t="n">
-        <v>3634</v>
+        <v>1500</v>
       </c>
       <c r="I192" s="138" t="n">
-        <v>4676</v>
+        <v>6416</v>
       </c>
       <c r="J192" s="139" t="n">
-        <v>1038.75</v>
+        <v>224.89</v>
       </c>
       <c r="K192" s="139" t="n">
-        <v>1038.23</v>
+        <v>220.56</v>
       </c>
       <c r="L192" s="236">
         <f>F192*(K192-J192)</f>
@@ -19751,31 +19751,31 @@
       <c r="C193" s="140" t="n"/>
       <c r="D193" s="137" t="inlineStr">
         <is>
-          <t>文曄(3036)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E193" s="138" t="n">
-        <v>352</v>
+        <v>500</v>
       </c>
       <c r="F193" s="138" t="n">
-        <v>67</v>
+        <v>259</v>
       </c>
       <c r="G193" s="138" t="n">
-        <v>7916</v>
+        <v>6135</v>
       </c>
       <c r="H193" s="138" t="n">
-        <v>1500</v>
+        <v>3188</v>
       </c>
       <c r="I193" s="138" t="n">
-        <v>6416</v>
+        <v>2947</v>
       </c>
       <c r="J193" s="139" t="n">
-        <v>224.89</v>
+        <v>122.71</v>
       </c>
       <c r="K193" s="139" t="n">
-        <v>223.85</v>
-      </c>
-      <c r="L193" s="236">
+        <v>123.09</v>
+      </c>
+      <c r="L193" s="235">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -19786,29 +19786,29 @@
       <c r="C194" s="140" t="n"/>
       <c r="D194" s="137" t="inlineStr">
         <is>
-          <t>旺宏(2337)</t>
+          <t>強茂(2481)</t>
         </is>
       </c>
       <c r="E194" s="138" t="n">
-        <v>130</v>
+        <v>332</v>
       </c>
       <c r="F194" s="138" t="n">
-        <v>76</v>
+        <v>18</v>
       </c>
       <c r="G194" s="138" t="n">
-        <v>6135</v>
+        <v>4589</v>
       </c>
       <c r="H194" s="138" t="n">
-        <v>3188</v>
+        <v>245</v>
       </c>
       <c r="I194" s="138" t="n">
-        <v>2947</v>
+        <v>4344</v>
       </c>
       <c r="J194" s="139" t="n">
-        <v>471.95</v>
+        <v>138.22</v>
       </c>
       <c r="K194" s="139" t="n">
-        <v>419.49</v>
+        <v>136.33</v>
       </c>
       <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
@@ -19821,29 +19821,29 @@
       <c r="C195" s="140" t="n"/>
       <c r="D195" s="137" t="inlineStr">
         <is>
-          <t>強茂(2481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E195" s="138" t="n">
-        <v>342</v>
+        <v>185</v>
       </c>
       <c r="F195" s="138" t="n">
-        <v>18</v>
+        <v>164</v>
       </c>
       <c r="G195" s="138" t="n">
-        <v>4589</v>
+        <v>3120</v>
       </c>
       <c r="H195" s="138" t="n">
-        <v>245</v>
+        <v>2775</v>
       </c>
       <c r="I195" s="138" t="n">
-        <v>4344</v>
+        <v>345</v>
       </c>
       <c r="J195" s="139" t="n">
-        <v>134.18</v>
+        <v>168.64</v>
       </c>
       <c r="K195" s="139" t="n">
-        <v>136.33</v>
+        <v>169.2</v>
       </c>
       <c r="L195" s="235">
         <f>F195*(K195-J195)</f>
@@ -19856,29 +19856,29 @@
       <c r="C196" s="140" t="n"/>
       <c r="D196" s="137" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E196" s="138" t="n">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="F196" s="138" t="n">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="G196" s="138" t="n">
-        <v>4494</v>
+        <v>2363</v>
       </c>
       <c r="H196" s="138" t="n">
-        <v>2448</v>
+        <v>1169</v>
       </c>
       <c r="I196" s="138" t="n">
-        <v>2046</v>
+        <v>1194</v>
       </c>
       <c r="J196" s="139" t="n">
-        <v>445</v>
+        <v>875.22</v>
       </c>
       <c r="K196" s="139" t="n">
-        <v>445</v>
+        <v>899.38</v>
       </c>
       <c r="L196" s="235">
         <f>F196*(K196-J196)</f>
@@ -19891,29 +19891,29 @@
       <c r="C197" s="140" t="n"/>
       <c r="D197" s="137" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E197" s="138" t="n">
-        <v>185</v>
+        <v>403</v>
       </c>
       <c r="F197" s="138" t="n">
-        <v>164</v>
+        <v>367</v>
       </c>
       <c r="G197" s="138" t="n">
-        <v>3120</v>
+        <v>1926</v>
       </c>
       <c r="H197" s="138" t="n">
-        <v>2775</v>
+        <v>1754</v>
       </c>
       <c r="I197" s="138" t="n">
-        <v>345</v>
+        <v>172</v>
       </c>
       <c r="J197" s="139" t="n">
-        <v>168.64</v>
+        <v>47.8</v>
       </c>
       <c r="K197" s="139" t="n">
-        <v>169.2</v>
+        <v>47.8</v>
       </c>
       <c r="L197" s="235">
         <f>F197*(K197-J197)</f>
@@ -19926,29 +19926,29 @@
       <c r="C198" s="140" t="n"/>
       <c r="D198" s="137" t="inlineStr">
         <is>
-          <t>環球晶(6488)</t>
+          <t>力成(6239)</t>
         </is>
       </c>
       <c r="E198" s="138" t="n">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="F198" s="138" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="G198" s="138" t="n">
-        <v>2363</v>
+        <v>1909</v>
       </c>
       <c r="H198" s="138" t="n">
-        <v>1169</v>
+        <v>1678</v>
       </c>
       <c r="I198" s="138" t="n">
-        <v>1194</v>
+        <v>231</v>
       </c>
       <c r="J198" s="139" t="n">
-        <v>875.22</v>
+        <v>258</v>
       </c>
       <c r="K198" s="139" t="n">
-        <v>899.38</v>
+        <v>258.12</v>
       </c>
       <c r="L198" s="235">
         <f>F198*(K198-J198)</f>
@@ -30578,7 +30578,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-06 00:38 TW | 19/19 success | 來源: 富邦19/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-06 01:29 TW | 19/19 success | 來源: 富邦19/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-08-06 22:57
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-08.xlsx
+++ b/data/reports/chip_radar_2026-08.xlsx
@@ -1765,7 +1765,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2330 / 6274 / 2308 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 11 檔: 1419, 1439, 1713 ...  |  訊號: 強偏多 (Q5 82.1%, hot=13)</t>
+          <t>💡 📌 一般共識 2330 / 6274 / 2308 (Q5 偏多但無 master 量爆 — alpha 未啟動)  |  避開 — 除權息 11 檔: 1419, 1439, 1713 ... | 明日恐處置 6 檔: 2059/2455/3037...  |  訊號: 強偏多 (Q5 82.1%, hot=13)</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
@@ -2298,13 +2298,13 @@
         </is>
       </c>
       <c r="L23" s="18" t="n">
-        <v>4686</v>
+        <v>5216</v>
       </c>
       <c r="M23" s="19" t="n">
         <v>8</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>33041</v>
+        <v>33571</v>
       </c>
     </row>
     <row r="24">
@@ -2529,23 +2529,23 @@
         <v>11</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="n">
+        <v>2206</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>張濬安</t>
         </is>
       </c>
-      <c r="H28" s="17" t="n">
+      <c r="J28" s="18" t="n">
         <v>1680</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="J28" s="18" t="n">
-        <v>1647</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>8</v>
       </c>
       <c r="N28" s="17" t="n">
-        <v>10228</v>
+        <v>10788</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="G31" s="257" t="n">
-        <v>-70.58412</v>
+        <v>-70.38218000000001</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="G32" s="259" t="n">
-        <v>0.1847289431673657</v>
+        <v>0.1849776296801424</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2681,11 +2681,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1333527</v>
+        <v>1341606</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>27.5%</t>
+          <t>27.6%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>22.9%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -3264,7 +3264,7 @@
         </is>
       </c>
       <c r="C65" s="33" t="n">
-        <v>1259132</v>
+        <v>1264701</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3291,7 +3291,7 @@
         <v>82320</v>
       </c>
       <c r="J65" s="214" t="n">
-        <v>0.3663949529663974</v>
+        <v>0.3647815356802178</v>
       </c>
     </row>
     <row r="66">
@@ -3741,7 +3741,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="B79" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260805)</t>
+          <t>▍ G. 注意股 (資料日 20260806)</t>
         </is>
       </c>
     </row>
@@ -3775,19 +3775,19 @@
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>039038</t>
+          <t>039037</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>富鼎統一6A購01</t>
+          <t>富鼎統一5A購01</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>1.85</v>
+        <v>1.69</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3798,19 +3798,19 @@
     <row r="82">
       <c r="B82" s="41" t="inlineStr">
         <is>
-          <t>053859</t>
+          <t>039038</t>
         </is>
       </c>
       <c r="C82" s="41" t="inlineStr">
         <is>
-          <t>強茂統一61購02</t>
+          <t>富鼎統一6A購01</t>
         </is>
       </c>
       <c r="D82" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E82" s="41" t="n">
-        <v>1.11</v>
+        <v>1.63</v>
       </c>
       <c r="F82" s="41" t="inlineStr">
         <is>
@@ -3821,19 +3821,19 @@
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>059816</t>
+          <t>040616</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>台虹凱基5A購02</t>
+          <t>華新科統一5A購01</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>1.14</v>
+        <v>6</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3844,19 +3844,19 @@
     <row r="84">
       <c r="B84" s="41" t="inlineStr">
         <is>
-          <t>068822</t>
+          <t>053859</t>
         </is>
       </c>
       <c r="C84" s="41" t="inlineStr">
         <is>
-          <t>富鼎統一69購01</t>
+          <t>強茂統一61購02</t>
         </is>
       </c>
       <c r="D84" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E84" s="41" t="n">
-        <v>0.84</v>
+        <v>1.09</v>
       </c>
       <c r="F84" s="41" t="inlineStr">
         <is>
@@ -3867,19 +3867,19 @@
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>071559</t>
+          <t>057151</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>強茂統一63購03</t>
+          <t>永光統一61購03</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
-        <v>0.64</v>
+        <v>0.9</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3890,230 +3890,230 @@
     <row r="86">
       <c r="B86" s="41" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>057514</t>
         </is>
       </c>
       <c r="C86" s="41" t="inlineStr">
         <is>
-          <t>亞德客-KY</t>
+          <t>強茂統一63購01</t>
         </is>
       </c>
       <c r="D86" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E86" s="41" t="n">
-        <v>1510</v>
+        <v>1.5</v>
       </c>
       <c r="F86" s="41" t="inlineStr">
         <is>
-          <t>33.06</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>059570</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>強茂凱基5B購03</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>9470</v>
+        <v>13.5</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>83.47</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" s="41" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>063447</t>
         </is>
       </c>
       <c r="C88" s="41" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>國巨統一74購01</t>
         </is>
       </c>
       <c r="D88" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E88" s="41" t="n">
-        <v>940</v>
+        <v>2.79</v>
       </c>
       <c r="F88" s="41" t="inlineStr">
         <is>
-          <t>42.44</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>064658</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>群創群益5A購04</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>5245</v>
+        <v>13</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>82.02</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="41" t="inlineStr">
         <is>
-          <t>2454</t>
+          <t>068822</t>
         </is>
       </c>
       <c r="C90" s="41" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>富鼎統一69購01</t>
         </is>
       </c>
       <c r="D90" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E90" s="41" t="n">
-        <v>4000</v>
+        <v>0.79</v>
       </c>
       <c r="F90" s="41" t="inlineStr">
         <is>
-          <t>66.06</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>2455</t>
+          <t>072318</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>全新</t>
+          <t>富鼎台新61購01</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>388</v>
+        <v>1.1</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>95.10</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" s="41" t="inlineStr">
         <is>
-          <t>2484</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="C92" s="41" t="inlineStr">
         <is>
-          <t>希華</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="D92" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E92" s="41" t="n">
-        <v>70.5</v>
+        <v>10100</v>
       </c>
       <c r="F92" s="41" t="inlineStr">
         <is>
-          <t>50.72</t>
+          <t>55.68</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2301</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>光寶科</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>969</v>
+        <v>252.5</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>64.51</t>
+          <t>29.53</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="41" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="C94" s="41" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="D94" s="41" t="n">
         <v>1</v>
       </c>
       <c r="E94" s="41" t="n">
-        <v>828</v>
+        <v>2410</v>
       </c>
       <c r="F94" s="41" t="inlineStr">
         <is>
-          <t>233.24</t>
+          <t>45.57</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>3443</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>創意</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>4390</v>
+        <v>5305</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>112.54</t>
+          <t>82.96</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
     <row r="115" ht="22" customHeight="1">
       <c r="B115" s="67" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 99 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 110 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -5210,9 +5210,9 @@
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="73" t="inlineStr">
-        <is>
-          <t>今日無處置股</t>
+      <c r="C33" s="71" t="inlineStr">
+        <is>
+          <t>明日恐處置 6 檔 (2059 / 2455 / 3037 ...)</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="247" t="inlineStr">
         <is>
-          <t>-71 億 淨買</t>
+          <t>-70 億 淨買</t>
         </is>
       </c>
     </row>
@@ -11891,7 +11891,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="106" t="inlineStr">
         <is>
-          <t>大牌分析師 近 75/75 交易日出手 3579 次 (600 檔), 風格分布: 隔日沖近似 32% / 當沖 14% / 留倉 54%, 漲停命中 4% (其中 🔒鎖漲停 3%), 前 5 大集中 24%, 長線部位 73% (67 檔), ⚠️ 處置股部位 11% (25 檔), 📦 連續囤貨 38 檔 (最長 13 天 009816, 3 檔仍 active)。 主軸: 📈 長線持有/高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 75/75 交易日出手 3579 次 (600 檔), 風格分布: 隔日沖近似 32% / 當沖 14% / 留倉 54%, 漲停命中 4% (其中 🔒鎖漲停 3%), 前 5 大集中 24%, 長線部位 73% (67 檔), ⚠️ 處置股部位 14% (41 檔), 📦 連續囤貨 38 檔 (最長 13 天 009816, 3 檔仍 active)。 主軸: 📈 長線持有/高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>
@@ -19451,7 +19451,7 @@
         </is>
       </c>
       <c r="E189" s="138" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F189" s="138" t="n">
         <v>5</v>
@@ -19466,7 +19466,7 @@
         <v>7646</v>
       </c>
       <c r="J189" s="139" t="n">
-        <v>991.9299999999999</v>
+        <v>979.98</v>
       </c>
       <c r="K189" s="139" t="n">
         <v>976.6</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="E191" s="138" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F191" s="138" t="n">
         <v>11</v>
@@ -19536,12 +19536,12 @@
         <v>4617</v>
       </c>
       <c r="J191" s="139" t="n">
-        <v>228.67</v>
+        <v>233.05</v>
       </c>
       <c r="K191" s="139" t="n">
         <v>230.73</v>
       </c>
-      <c r="L191" s="235">
+      <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -19657,29 +19657,29 @@
       <c r="C195" s="140" t="n"/>
       <c r="D195" s="137" t="inlineStr">
         <is>
-          <t>景碩(3189)</t>
+          <t>力積電(6770)</t>
         </is>
       </c>
       <c r="E195" s="138" t="n">
-        <v>30</v>
+        <v>393</v>
       </c>
       <c r="F195" s="138" t="n">
-        <v>22</v>
+        <v>309</v>
       </c>
       <c r="G195" s="138" t="n">
-        <v>2566</v>
+        <v>2617</v>
       </c>
       <c r="H195" s="138" t="n">
-        <v>1917</v>
+        <v>2058</v>
       </c>
       <c r="I195" s="138" t="n">
-        <v>649</v>
+        <v>559</v>
       </c>
       <c r="J195" s="139" t="n">
-        <v>855.4</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="K195" s="139" t="n">
-        <v>871.3200000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="L195" s="235">
         <f>F195*(K195-J195)</f>
@@ -19692,29 +19692,29 @@
       <c r="C196" s="140" t="n"/>
       <c r="D196" s="137" t="inlineStr">
         <is>
-          <t>欣興(3037)</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E196" s="138" t="n">
+        <v>30</v>
+      </c>
+      <c r="F196" s="138" t="n">
         <v>22</v>
       </c>
-      <c r="F196" s="138" t="n">
-        <v>19</v>
-      </c>
       <c r="G196" s="138" t="n">
-        <v>2108</v>
+        <v>2566</v>
       </c>
       <c r="H196" s="138" t="n">
-        <v>1833</v>
+        <v>1917</v>
       </c>
       <c r="I196" s="138" t="n">
-        <v>275</v>
+        <v>649</v>
       </c>
       <c r="J196" s="139" t="n">
-        <v>958.27</v>
+        <v>855.4</v>
       </c>
       <c r="K196" s="139" t="n">
-        <v>964.84</v>
+        <v>871.3200000000001</v>
       </c>
       <c r="L196" s="235">
         <f>F196*(K196-J196)</f>
@@ -19727,29 +19727,29 @@
       <c r="C197" s="140" t="n"/>
       <c r="D197" s="137" t="inlineStr">
         <is>
-          <t>穩懋(3105)</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E197" s="138" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="F197" s="138" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="G197" s="138" t="n">
-        <v>2099</v>
+        <v>2108</v>
       </c>
       <c r="H197" s="138" t="n">
-        <v>1795</v>
+        <v>1833</v>
       </c>
       <c r="I197" s="138" t="n">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="J197" s="139" t="n">
-        <v>381.58</v>
+        <v>958.27</v>
       </c>
       <c r="K197" s="139" t="n">
-        <v>381.85</v>
+        <v>964.84</v>
       </c>
       <c r="L197" s="235">
         <f>F197*(K197-J197)</f>
@@ -19762,29 +19762,29 @@
       <c r="C198" s="140" t="n"/>
       <c r="D198" s="137" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>穩懋(3105)</t>
         </is>
       </c>
       <c r="E198" s="138" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="F198" s="138" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="G198" s="138" t="n">
-        <v>1766</v>
+        <v>2099</v>
       </c>
       <c r="H198" s="138" t="n">
-        <v>1280</v>
+        <v>1795</v>
       </c>
       <c r="I198" s="138" t="n">
-        <v>486</v>
+        <v>304</v>
       </c>
       <c r="J198" s="139" t="n">
-        <v>569.6799999999999</v>
+        <v>381.58</v>
       </c>
       <c r="K198" s="139" t="n">
-        <v>581.95</v>
+        <v>381.85</v>
       </c>
       <c r="L198" s="235">
         <f>F198*(K198-J198)</f>
@@ -30271,7 +30271,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-08-06 21:36 TW | 11/11 success | 來源: 富邦11/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-08-06 22:57 TW | 11/11 success | 來源: 富邦11/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>